<commit_message>
Atualiza dashboard Giuriolo: docs/historico_giuriolo.xlsx
</commit_message>
<xml_diff>
--- a/docs/historico_giuriolo.xlsx
+++ b/docs/historico_giuriolo.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR20"/>
+  <dimension ref="A1:AS20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -644,6 +644,11 @@
           <t>2026-04-07</t>
         </is>
       </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -778,6 +783,9 @@
         <v>4420</v>
       </c>
       <c r="AR2" t="n">
+        <v>4442</v>
+      </c>
+      <c r="AS2" t="n">
         <v>4442</v>
       </c>
     </row>
@@ -886,6 +894,9 @@
       <c r="AR3" t="n">
         <v>559</v>
       </c>
+      <c r="AS3" t="n">
+        <v>559</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -1022,6 +1033,9 @@
       <c r="AR4" t="n">
         <v>1788</v>
       </c>
+      <c r="AS4" t="n">
+        <v>1788</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -1156,7 +1170,10 @@
         <v>658</v>
       </c>
       <c r="AR5" t="n">
-        <v>694</v>
+        <v>690</v>
+      </c>
+      <c r="AS5" t="n">
+        <v>695</v>
       </c>
     </row>
     <row r="6">
@@ -1264,6 +1281,9 @@
       <c r="AR6" t="n">
         <v>2</v>
       </c>
+      <c r="AS6" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -1398,6 +1418,9 @@
         <v>81</v>
       </c>
       <c r="AR7" t="n">
+        <v>49</v>
+      </c>
+      <c r="AS7" t="n">
         <v>48</v>
       </c>
     </row>
@@ -1506,6 +1529,9 @@
       <c r="AR8" t="n">
         <v>19</v>
       </c>
+      <c r="AS8" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -1612,6 +1638,9 @@
       <c r="AR9" t="n">
         <v>2</v>
       </c>
+      <c r="AS9" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -1748,6 +1777,9 @@
       <c r="AR10" t="n">
         <v>1272</v>
       </c>
+      <c r="AS10" t="n">
+        <v>1272</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
@@ -1882,7 +1914,10 @@
         <v>62</v>
       </c>
       <c r="AR11" t="n">
-        <v>58</v>
+        <v>61</v>
+      </c>
+      <c r="AS11" t="n">
+        <v>57</v>
       </c>
     </row>
     <row r="12">
@@ -2020,6 +2055,9 @@
       <c r="AR12" t="n">
         <v>1</v>
       </c>
+      <c r="AS12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
@@ -2153,7 +2191,10 @@
       <c r="AQ13" t="n">
         <v>1</v>
       </c>
-      <c r="AR13" t="inlineStr"/>
+      <c r="AR13" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
@@ -2287,7 +2328,10 @@
       <c r="AQ14" t="n">
         <v>79</v>
       </c>
-      <c r="AR14" t="inlineStr"/>
+      <c r="AR14" t="n">
+        <v>47</v>
+      </c>
+      <c r="AS14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
@@ -2424,6 +2468,9 @@
       <c r="AR15" t="n">
         <v>64</v>
       </c>
+      <c r="AS15" t="n">
+        <v>64</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
@@ -2560,6 +2607,9 @@
       <c r="AR16" t="n">
         <v>864</v>
       </c>
+      <c r="AS16" t="n">
+        <v>864</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
@@ -2694,6 +2744,9 @@
         <v>1524</v>
       </c>
       <c r="AR17" t="n">
+        <v>1524</v>
+      </c>
+      <c r="AS17" t="n">
         <v>1536</v>
       </c>
     </row>
@@ -2830,7 +2883,10 @@
         <v>6.5</v>
       </c>
       <c r="AR18" t="n">
-        <v>6.37</v>
+        <v>6.372093023255814</v>
+      </c>
+      <c r="AS18" t="n">
+        <v>6.23</v>
       </c>
     </row>
     <row r="19">
@@ -2966,7 +3022,10 @@
         <v>133.0769230769231</v>
       </c>
       <c r="AR19" t="n">
-        <v>135.59</v>
+        <v>135.5912408759124</v>
+      </c>
+      <c r="AS19" t="n">
+        <v>138.74</v>
       </c>
     </row>
     <row r="20">
@@ -3187,7 +3246,12 @@
       </c>
       <c r="AR20" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="AS20" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>

</xml_diff>